<commit_message>
Extend Dictionary tab for DCAT-AP-CH metadata
</commit_message>
<xml_diff>
--- a/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
+++ b/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
@@ -2910,7 +2910,11 @@
       <c r="J11" s="77" t="n"/>
       <c r="K11" s="78" t="n"/>
       <c r="L11" s="73" t="n"/>
-      <c r="M11" s="79" t="n"/>
+      <c r="M11" s="79" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeSegmentFLEXIBLESEGMENT</t>
+        </is>
+      </c>
       <c r="N11" s="80" t="n"/>
       <c r="O11" s="80" t="n"/>
       <c r="P11" s="81" t="n"/>
@@ -2936,7 +2940,11 @@
       <c r="J12" s="91" t="n"/>
       <c r="K12" s="92" t="n"/>
       <c r="L12" s="88" t="n"/>
-      <c r="M12" s="93" t="n"/>
+      <c r="M12" s="93" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingBEND</t>
+        </is>
+      </c>
       <c r="N12" s="94" t="n"/>
       <c r="O12" s="94" t="n"/>
       <c r="P12" s="95" t="n"/>
@@ -2962,7 +2970,11 @@
       <c r="J13" s="91" t="n"/>
       <c r="K13" s="92" t="n"/>
       <c r="L13" s="88" t="n"/>
-      <c r="M13" s="93" t="n"/>
+      <c r="M13" s="93" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingJUNCTION</t>
+        </is>
+      </c>
       <c r="N13" s="94" t="n"/>
       <c r="O13" s="94" t="n"/>
       <c r="P13" s="95" t="n"/>
@@ -2988,7 +3000,11 @@
       <c r="J14" s="91" t="n"/>
       <c r="K14" s="92" t="n"/>
       <c r="L14" s="88" t="n"/>
-      <c r="M14" s="100" t="n"/>
+      <c r="M14" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingTRANSITION</t>
+        </is>
+      </c>
       <c r="N14" s="94" t="n"/>
       <c r="O14" s="94" t="n"/>
       <c r="P14" s="95" t="n"/>
@@ -3014,7 +3030,11 @@
       <c r="J15" s="91" t="n"/>
       <c r="K15" s="92" t="n"/>
       <c r="L15" s="88" t="n"/>
-      <c r="M15" s="100" t="n"/>
+      <c r="M15" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingTRANSITION</t>
+        </is>
+      </c>
       <c r="N15" s="94" t="n"/>
       <c r="O15" s="94" t="n"/>
       <c r="P15" s="95" t="n"/>
@@ -3040,7 +3060,11 @@
       <c r="J16" s="91" t="n"/>
       <c r="K16" s="92" t="n"/>
       <c r="L16" s="88" t="n"/>
-      <c r="M16" s="100" t="n"/>
+      <c r="M16" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingBEND</t>
+        </is>
+      </c>
       <c r="N16" s="94" t="n"/>
       <c r="O16" s="94" t="n"/>
       <c r="P16" s="95" t="n"/>
@@ -3066,7 +3090,11 @@
       <c r="J17" s="91" t="n"/>
       <c r="K17" s="92" t="n"/>
       <c r="L17" s="88" t="n"/>
-      <c r="M17" s="100" t="n"/>
+      <c r="M17" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingCONNECTOR</t>
+        </is>
+      </c>
       <c r="N17" s="94" t="n"/>
       <c r="O17" s="94" t="n"/>
       <c r="P17" s="95" t="n"/>
@@ -3092,7 +3120,11 @@
       <c r="J18" s="91" t="n"/>
       <c r="K18" s="92" t="n"/>
       <c r="L18" s="88" t="n"/>
-      <c r="M18" s="100" t="n"/>
+      <c r="M18" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcPipeFittingCONNECTOR</t>
+        </is>
+      </c>
       <c r="N18" s="94" t="n"/>
       <c r="O18" s="94" t="n"/>
       <c r="P18" s="95" t="n"/>
@@ -3118,7 +3150,11 @@
       <c r="J19" s="91" t="n"/>
       <c r="K19" s="92" t="n"/>
       <c r="L19" s="88" t="n"/>
-      <c r="M19" s="100" t="n"/>
+      <c r="M19" s="100" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/class/IfcHeatExchanger</t>
+        </is>
+      </c>
       <c r="N19" s="94" t="n"/>
       <c r="O19" s="94" t="n"/>
       <c r="P19" s="95" t="n"/>
@@ -6361,7 +6397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:O61"/>
+  <dimension ref="B2:O61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col width="1.7109375" customWidth="1" style="175" min="1" max="1"/>
@@ -6937,7 +6973,11 @@
       <c r="O33" s="197" t="n"/>
     </row>
     <row r="34" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B34" s="199" t="n"/>
+      <c r="B34" s="199" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/IsExternal</t>
+        </is>
+      </c>
       <c r="C34" s="199" t="n"/>
       <c r="D34" s="199" t="n"/>
       <c r="E34" s="199" t="n"/>
@@ -6953,7 +6993,11 @@
       <c r="O34" s="197" t="n"/>
     </row>
     <row r="35" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B35" s="202" t="n"/>
+      <c r="B35" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyType</t>
+        </is>
+      </c>
       <c r="C35" s="199" t="n"/>
       <c r="D35" s="199" t="n"/>
       <c r="E35" s="199" t="n"/>
@@ -6985,7 +7029,11 @@
       <c r="O36" s="197" t="n"/>
     </row>
     <row r="37" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B37" s="199" t="n"/>
+      <c r="B37" s="199" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyNumberPeak</t>
+        </is>
+      </c>
       <c r="C37" s="199" t="n"/>
       <c r="D37" s="199" t="n"/>
       <c r="E37" s="199" t="n"/>
@@ -7001,7 +7049,11 @@
       <c r="O37" s="197" t="n"/>
     </row>
     <row r="38" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B38" s="202" t="n"/>
+      <c r="B38" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/OccupancyNumber</t>
+        </is>
+      </c>
       <c r="C38" s="199" t="n"/>
       <c r="D38" s="199" t="n"/>
       <c r="E38" s="199" t="n"/>
@@ -7017,7 +7069,11 @@
       <c r="O38" s="197" t="n"/>
     </row>
     <row r="39" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B39" s="202" t="n"/>
+      <c r="B39" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/FloorCovering</t>
+        </is>
+      </c>
       <c r="C39" s="199" t="n"/>
       <c r="D39" s="199" t="n"/>
       <c r="E39" s="199" t="n"/>
@@ -7033,7 +7089,11 @@
       <c r="O39" s="197" t="n"/>
     </row>
     <row r="40" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B40" s="202" t="n"/>
+      <c r="B40" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/WallCovering</t>
+        </is>
+      </c>
       <c r="C40" s="199" t="n"/>
       <c r="D40" s="199" t="n"/>
       <c r="E40" s="199" t="n"/>
@@ -7049,7 +7109,11 @@
       <c r="O40" s="197" t="n"/>
     </row>
     <row r="41" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B41" s="202" t="n"/>
+      <c r="B41" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/CeilingCovering</t>
+        </is>
+      </c>
       <c r="C41" s="199" t="n"/>
       <c r="D41" s="199" t="n"/>
       <c r="E41" s="199" t="n"/>
@@ -7065,7 +7129,11 @@
       <c r="O41" s="197" t="n"/>
     </row>
     <row r="42" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B42" s="202" t="n"/>
+      <c r="B42" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NaturalVentilation</t>
+        </is>
+      </c>
       <c r="C42" s="199" t="n"/>
       <c r="D42" s="199" t="n"/>
       <c r="E42" s="199" t="n"/>
@@ -7081,7 +7149,11 @@
       <c r="O42" s="197" t="n"/>
     </row>
     <row r="43" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B43" s="202" t="n"/>
+      <c r="B43" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NaturalVentilationRate</t>
+        </is>
+      </c>
       <c r="C43" s="199" t="n"/>
       <c r="D43" s="199" t="n"/>
       <c r="E43" s="199" t="n"/>
@@ -7097,7 +7169,11 @@
       <c r="O43" s="197" t="n"/>
     </row>
     <row r="44" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B44" s="202" t="n"/>
+      <c r="B44" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/MechanicalVentilation</t>
+        </is>
+      </c>
       <c r="C44" s="199" t="n"/>
       <c r="D44" s="199" t="n"/>
       <c r="E44" s="199" t="n"/>
@@ -7113,7 +7189,11 @@
       <c r="O44" s="197" t="n"/>
     </row>
     <row r="45" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B45" s="202" t="n"/>
+      <c r="B45" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/MechanicalVentilationRate</t>
+        </is>
+      </c>
       <c r="C45" s="199" t="n"/>
       <c r="D45" s="199" t="n"/>
       <c r="E45" s="199" t="n"/>
@@ -7129,7 +7209,11 @@
       <c r="O45" s="197" t="n"/>
     </row>
     <row r="46" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B46" s="202" t="n"/>
+      <c r="B46" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/AirConditioning</t>
+        </is>
+      </c>
       <c r="C46" s="199" t="n"/>
       <c r="D46" s="199" t="n"/>
       <c r="E46" s="199" t="n"/>
@@ -7145,7 +7229,11 @@
       <c r="O46" s="197" t="n"/>
     </row>
     <row r="47" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B47" s="202" t="n"/>
+      <c r="B47" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/TemperatureSetPoint</t>
+        </is>
+      </c>
       <c r="C47" s="199" t="n"/>
       <c r="D47" s="199" t="n"/>
       <c r="E47" s="199" t="n"/>
@@ -7161,7 +7249,11 @@
       <c r="O47" s="197" t="n"/>
     </row>
     <row r="48" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B48" s="202" t="n"/>
+      <c r="B48" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/HumiditySetPoint</t>
+        </is>
+      </c>
       <c r="C48" s="199" t="n"/>
       <c r="D48" s="199" t="n"/>
       <c r="E48" s="199" t="n"/>
@@ -7177,7 +7269,11 @@
       <c r="O48" s="197" t="n"/>
     </row>
     <row r="49" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B49" s="202" t="n"/>
+      <c r="B49" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/FireExit</t>
+        </is>
+      </c>
       <c r="C49" s="199" t="n"/>
       <c r="D49" s="199" t="n"/>
       <c r="E49" s="199" t="n"/>
@@ -7193,7 +7289,11 @@
       <c r="O49" s="197" t="n"/>
     </row>
     <row r="50" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B50" s="202" t="n"/>
+      <c r="B50" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/GrossFloorArea</t>
+        </is>
+      </c>
       <c r="C50" s="199" t="n"/>
       <c r="D50" s="199" t="n"/>
       <c r="E50" s="199" t="n"/>
@@ -7209,7 +7309,11 @@
       <c r="O50" s="197" t="n"/>
     </row>
     <row r="51" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B51" s="202" t="n"/>
+      <c r="B51" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/GrossVolume</t>
+        </is>
+      </c>
       <c r="C51" s="199" t="n"/>
       <c r="D51" s="199" t="n"/>
       <c r="E51" s="199" t="n"/>
@@ -7225,7 +7329,11 @@
       <c r="O51" s="197" t="n"/>
     </row>
     <row r="52" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B52" s="202" t="n"/>
+      <c r="B52" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NetFloorArea</t>
+        </is>
+      </c>
       <c r="C52" s="199" t="n"/>
       <c r="D52" s="199" t="n"/>
       <c r="E52" s="199" t="n"/>
@@ -7241,7 +7349,11 @@
       <c r="O52" s="197" t="n"/>
     </row>
     <row r="53" ht="15" customFormat="1" customHeight="1" s="203">
-      <c r="B53" s="202" t="n"/>
+      <c r="B53" s="202" t="inlineStr">
+        <is>
+          <t>https://identifier.buildingsmart.org/uri/buildingsmart/ifc/4.3/prop/NetVolume</t>
+        </is>
+      </c>
       <c r="C53" s="199" t="n"/>
       <c r="D53" s="199" t="n"/>
       <c r="E53" s="199" t="n"/>
@@ -7300,7 +7412,6 @@
       <c r="N56" s="198" t="n"/>
       <c r="O56" s="197" t="n"/>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="G58" s="196" t="n"/>
       <c r="H58" s="195" t="n"/>
@@ -7390,7 +7501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7584,61 +7695,625 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LifecycleStatus</t>
+        </is>
+      </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fill business metadata only. Keep stable identifiers/URIs consistent. DictionaryCode is required and should be short, stable, and namespace-safe.</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Governance state, e.g. draft/published/deprecated — adms:status / lifecycle metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Owner / Publisher</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>KBOB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Owning or publishing organization — dct:publisher / i14y publisher</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Description (DE)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nationaler Datenkatalog für strukturierte Merkmale, Klassen und semantische Datenvorlagen im KBOB-/HE-SEM-Kontext.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Dictionary description in German — dct:description@de</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Description (FR)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dictionary description in French — dct:description@fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Description (EN)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Dictionary description in English — dct:description@en</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ContactEmail</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>kbob@bbl.admin.ch</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Contact mailbox for maintenance/governance — dcat:contactPoint / i14y contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PrimaryLanguage</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Primary language of the metadata/content — dct:language (main)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MetadataLanguages</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Additional metadata languages; use delimited list if needed — dct:language</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ReleaseDate</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Initial public release date — dct:issued</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ModifiedDate</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Last metadata/content update date — dct:modified</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Keywords (DE)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>German keywords/tags — dcat:keyword@de</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Keywords (FR)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>French keywords/tags — dcat:keyword@fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Keywords (EN)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>English keywords/tags — dcat:keyword@en</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AccessRights</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Access rights / visibility statement — dct:accessRights</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>eCH_Theme</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Swiss eCH thematic classification / topic category</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SpatialCoverage</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Geographic scope or covered territory — dct:spatial</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TemporalCoverage</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Covered time period / validity period — dct:temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DocumentationURLs</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Supporting documentation links; use delimited list if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RelatedResourceURLs</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Related datasets/resources links; use delimited list if needed — dct:relation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ApplicableLegislation</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Applicable legal basis / legislation references</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Human-readable license name — dct:license</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LicenseUrl</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Resolvable license URI/URL — dct:license</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SPARQL_Endpoint</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SPARQL endpoint URL for published graph access</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>TTL_Download_URL</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Download URL for Turtle/RDF serialization — dcat:distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>JSON_Download_URL</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Download URL for JSON/JSON-LD serialization — dcat:distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>MoreInfoUrl</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Landing page / more information URL — rdfs:seeAlso / dcat:landingPage</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ConformsTo_ISO23386</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Conformance flag or statement for ISO 23386 — dct:conformsTo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ConformsTo_ISO12006_3</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Conformance flag or statement for ISO 12006-3 — dct:conformsTo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ConformsTo_DCAT_AP_CH</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Conformance flag or statement for DCAT-AP CH — dct:conformsTo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QualityAssuranceProcedure</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Short QA / review procedure description</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>QualityAssuranceProcedureUrl</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>URL to QA procedure, review checklist, or governance page</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>VersionNotes (DE)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>German release/change notes — adms:versionNotes@de</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>VersionNotes (FR)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>French release/change notes — adms:versionNotes@fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>VersionNotes (EN)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>English release/change notes — adms:versionNotes@en</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Fill business metadata only. Keep stable identifiers/URIs consistent. Use these rows to capture governance and DCAT/i14y publication metadata in a structured way.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
           <t>Guide</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>System uses this metadata to build IRIs and governance context. LifecycleStatus: required. List-based validation. DictionaryVersion: required. Regex-based validation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>System uses this metadata to build IRIs, governance context, and publication/export mappings. DictionaryCode, DictionaryVersion, DictionaryUri, and LifecycleStatus are formal field rows; add publication URLs and conformance statements where available.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7650,7 +8325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7742,7 +8417,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Split dictionary core/public metadata tabs
</commit_message>
<xml_diff>
--- a/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
+++ b/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Merkmale_Merkmalsgruppen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dokumente_Dokumentgruppen" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KlassenMerkmal" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConceptRelation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary core" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary public" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ConceptRelation" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -7507,7 +7508,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>HE-SEM Data Dictionary — Container Metadata (Tab 1)</t>
+          <t>HE-SEM Data Dictionary — Core Metadata (mandatory authoring block)</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7603,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>rdfs:label@de / dct:title@de</t>
+          <t>Core authoring title in German — minimal DCAT/i14y anchor</t>
         </is>
       </c>
     </row>
@@ -7619,12 +7620,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>REQUIRED</t>
+          <t>OPTIONAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>rdfs:label@fr / dct:title@fr</t>
+          <t>Optional multilingual title support</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7647,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>rdfs:label@en / dct:title@en</t>
+          <t>Optional multilingual title support</t>
         </is>
       </c>
     </row>
@@ -7695,625 +7696,111 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>LifecycleStatus</t>
-        </is>
-      </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Preview</t>
+          <t>Minimal mandatory block: validator currently enforces only these core fields for DCAT/i14y baseline compatibility.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>REQUIRED</t>
+          <t>Guide</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Governance state, e.g. draft/published/deprecated — adms:status / lifecycle metadata</t>
+          <t>Private organisations may keep only this tab and delete Dictionary public.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Owner / Publisher</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>KBOB</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Owning or publishing organization — dct:publisher / i14y publisher</t>
+          <t>── GOVERNANCE ──</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Description (DE)</t>
+          <t>LifecycleStatus</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nationaler Datenkatalog für strukturierte Merkmale, Klassen und semantische Datenvorlagen im KBOB-/HE-SEM-Kontext.</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>OPTIONAL</t>
+          <t>REQUIRED</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dictionary description in German — dct:description@de</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Description (FR)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Dictionary description in French — dct:description@fr</t>
-        </is>
-      </c>
-    </row>
+          <t>Governance state used to derive i14y registration status</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Description (EN)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Dictionary description in English — dct:description@en</t>
+          <t>LEGEND:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ContactEmail</t>
+          <t>REQUIRED</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>kbob@bbl.admin.ch</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Contact mailbox for maintenance/governance — dcat:contactPoint / i14y contact</t>
+          <t>Must be filled before validation/export</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PrimaryLanguage</t>
+          <t>OPTIONAL</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>de</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Primary language of the metadata/content — dct:language (main)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>MetadataLanguages</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Additional metadata languages; use delimited list if needed — dct:language</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ReleaseDate</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Initial public release date — dct:issued</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ModifiedDate</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Last metadata/content update date — dct:modified</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Keywords (DE)</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>German keywords/tags — dcat:keyword@de</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Keywords (FR)</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>French keywords/tags — dcat:keyword@fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Keywords (EN)</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>English keywords/tags — dcat:keyword@en</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>AccessRights</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Access rights / visibility statement — dct:accessRights</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>eCH_Theme</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Swiss eCH thematic classification / topic category</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>SpatialCoverage</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Geographic scope or covered territory — dct:spatial</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>TemporalCoverage</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Covered time period / validity period — dct:temporal</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>DocumentationURLs</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Supporting documentation links; use delimited list if needed</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>RelatedResourceURLs</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Related datasets/resources links; use delimited list if needed — dct:relation</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>ApplicableLegislation</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Applicable legal basis / legislation references</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>License</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Human-readable license name — dct:license</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>LicenseUrl</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Resolvable license URI/URL — dct:license</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SPARQL_Endpoint</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>SPARQL endpoint URL for published graph access</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>TTL_Download_URL</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Download URL for Turtle/RDF serialization — dcat:distribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>JSON_Download_URL</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Download URL for JSON/JSON-LD serialization — dcat:distribution</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>MoreInfoUrl</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Landing page / more information URL — rdfs:seeAlso / dcat:landingPage</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ConformsTo_ISO23386</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Conformance flag or statement for ISO 23386 — dct:conformsTo</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>ConformsTo_ISO12006_3</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Conformance flag or statement for ISO 12006-3 — dct:conformsTo</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>ConformsTo_DCAT_AP_CH</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Conformance flag or statement for DCAT-AP CH — dct:conformsTo</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>QualityAssuranceProcedure</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Short QA / review procedure description</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>QualityAssuranceProcedureUrl</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>URL to QA procedure, review checklist, or governance page</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>VersionNotes (DE)</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>German release/change notes — adms:versionNotes@de</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>VersionNotes (FR)</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>French release/change notes — adms:versionNotes@fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>VersionNotes (EN)</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>English release/change notes — adms:versionNotes@en</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Fill business metadata only. Keep stable identifiers/URIs consistent. Use these rows to capture governance and DCAT/i14y publication metadata in a structured way.</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>System uses this metadata to build IRIs, governance context, and publication/export mappings. DictionaryCode, DictionaryVersion, DictionaryUri, and LifecycleStatus are formal field rows; add publication URLs and conformance statements where available.</t>
-        </is>
-      </c>
-    </row>
+          <t>Fill if available</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8325,6 +7812,749 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>HE-SEM Data Dictionary — Public Metadata (optional extended publication block)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Notes / Maps to</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>── GOVERNANCE / PUBLISHING ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Owner / Publisher</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KBOB</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>REQUIRED WHEN USED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>dct:publisher / i14y publisher mapping</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ContactEmail</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>kbob@bbl.admin.ch</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REQUIRED WHEN USED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>dcat:contactPoint / i14y contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Description (DE)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Nationaler Datenkatalog für strukturierte Merkmale, Klassen und semantische Datenvorlagen im KBOB-/HE-SEM-Kontext.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>REQUIRED WHEN USED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>dct:description@de</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Description (FR)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dct:description@fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Description (EN)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>dct:description@en</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PrimaryLanguage</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>REQUIRED WHEN USED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Primary metadata/content language</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MetadataLanguages</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Additional metadata languages; delimited list allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ReleaseDate</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>dct:issued — format YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ModifiedDate</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>dct:modified — format YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>QualityAssuranceProcedure</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ISO 23386:2020</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>dct:conformsTo — QA method label</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>QualityAssuranceProcedureUrl</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.iso.org/standard/75401.html</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>URL to QA procedure</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>── DISCOVERY / CATALOG METADATA ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Keywords (DE)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>German keywords/tags — dcat:keyword@de</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Keywords (FR)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>French keywords/tags — dcat:keyword@fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Keywords (EN)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>English keywords/tags — dcat:keyword@en</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AccessRights</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Access rights / visibility statement — dct:accessRights</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>eCH_Theme</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Swiss eCH thematic classification / topic category</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SpatialCoverage</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Geographic scope or covered territory — dct:spatial</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TemporalCoverage</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Covered time period / validity period — dct:temporal</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DocumentationURLs</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Supporting documentation links; delimited list allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RelatedResourceURLs</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Related datasets/resources links — dct:relation</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ApplicableLegislation</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Applicable legal basis / legislation references</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>── LICENSING ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>License</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Human-readable license name — dct:license</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LicenseUrl</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Resolvable license URI/URL — dct:license</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>── TECHNICAL ENDPOINTS ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SPARQL_Endpoint</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SPARQL endpoint URL for published graph access</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TTL_Download_URL</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Download URL for Turtle/RDF serialization — dcat:distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>JSON_Download_URL</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Download URL for JSON/JSON-LD serialization — dcat:distribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MoreInfoUrl</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Landing page / homepage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>── STANDARDS ALIGNMENT ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ConformsTo_ISO23386</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://www.iso.org/standard/75401.html</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>dct:conformsTo — property methodology</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ConformsTo_ISO12006_3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://www.iso.org/standard/57834.html</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>dct:conformsTo — data dictionary meta-model</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ConformsTo_DCAT_AP_CH</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://dcat-ap.ch/releases/v3/3.0.0.html</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>dct:conformsTo — Swiss catalog profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>VersionNotes (DE)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Release/version notes in German</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>VersionNotes (FR)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Release/version notes in French</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>VersionNotes (EN)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Release/version notes in English</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Optional extended block: not part of the current minimal validator gate unless this tab is present/used; when filled, SchemaForge should consume it for publication payloads.</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Public organisations can keep and fill this tab; private organisations can delete it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LEGEND:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>REQUIRED WHEN USED</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Must be filled once Dictionary public is used for publication metadata</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Fill if available</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Make split-tab test workbook empty authoring template
</commit_message>
<xml_diff>
--- a/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
+++ b/templates/HE_DD_Strukturvorlagev0.1__authoring-guidance_test.xlsx
@@ -7502,7 +7502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7547,11 +7547,6 @@
           <t>OrganizationCode</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>kbob</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>REQUIRED</t>
@@ -7569,11 +7564,6 @@
           <t>DictionaryCode</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DD_FM</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>REQUIRED</t>
@@ -7591,11 +7581,6 @@
           <t>DictionaryName (DE)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>KBOB Datenkatalog</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>REQUIRED</t>
@@ -7613,11 +7598,6 @@
           <t>DictionaryName (FR)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Catalogue de données DD_FM</t>
-        </is>
-      </c>
       <c r="C7" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -7635,11 +7615,6 @@
           <t>DictionaryName (EN)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>KBOB Data Dictionary</t>
-        </is>
-      </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -7657,11 +7632,6 @@
           <t>DictionaryVersion</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>REQUIRED</t>
@@ -7679,11 +7649,6 @@
           <t>DictionaryUri</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>https://www.kbob.admin.ch/dictionary/kbob</t>
-        </is>
-      </c>
       <c r="C10" t="inlineStr">
         <is>
           <t>REQUIRED</t>
@@ -7723,11 +7688,6 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>LifecycleStatus</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Preview</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -7773,34 +7733,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7812,7 +7744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7857,11 +7789,6 @@
           <t>Owner / Publisher</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>KBOB</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>REQUIRED WHEN USED</t>
@@ -7879,11 +7806,6 @@
           <t>ContactEmail</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>kbob@bbl.admin.ch</t>
-        </is>
-      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>REQUIRED WHEN USED</t>
@@ -7901,11 +7823,6 @@
           <t>Description (DE)</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Nationaler Datenkatalog für strukturierte Merkmale, Klassen und semantische Datenvorlagen im KBOB-/HE-SEM-Kontext.</t>
-        </is>
-      </c>
       <c r="C6" t="inlineStr">
         <is>
           <t>REQUIRED WHEN USED</t>
@@ -7957,11 +7874,6 @@
           <t>PrimaryLanguage</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>de</t>
-        </is>
-      </c>
       <c r="C9" t="inlineStr">
         <is>
           <t>REQUIRED WHEN USED</t>
@@ -8030,11 +7942,6 @@
           <t>QualityAssuranceProcedure</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>ISO 23386:2020</t>
-        </is>
-      </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -8052,11 +7959,6 @@
           <t>QualityAssuranceProcedureUrl</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>https://www.iso.org/standard/75401.html</t>
-        </is>
-      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -8374,11 +8276,6 @@
           <t>ConformsTo_ISO23386</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>https://www.iso.org/standard/75401.html</t>
-        </is>
-      </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -8396,11 +8293,6 @@
           <t>ConformsTo_ISO12006_3</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>https://www.iso.org/standard/57834.html</t>
-        </is>
-      </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
@@ -8416,11 +8308,6 @@
       <c r="A37" t="inlineStr">
         <is>
           <t>ConformsTo_DCAT_AP_CH</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>https://dcat-ap.ch/releases/v3/3.0.0.html</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -8534,16 +8421,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>